<commit_message>
fix: loop between variables of CD
</commit_message>
<xml_diff>
--- a/Experiment3/Workspace/Models/notebooks/sweep_outputs/comparison_chains_full_metrics.xlsx
+++ b/Experiment3/Workspace/Models/notebooks/sweep_outputs/comparison_chains_full_metrics.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ4"/>
+  <dimension ref="A1:AJ7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -618,17 +618,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>multiple_none_mse_plain_gat</t>
+          <t>single_none_mse_plain_gat</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1_multi_relation_baseline</t>
+          <t>0_single_relation_baseline</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>multiple</t>
+          <t>single</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -655,73 +655,73 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>3092.066526889801</v>
+        <v>1173.004513978958</v>
       </c>
       <c r="K2" t="n">
-        <v>0.5412698412698413</v>
+        <v>0.5904761904761904</v>
       </c>
       <c r="L2" t="n">
-        <v>0.0869980292447283</v>
+        <v>0.06459361888690729</v>
       </c>
       <c r="M2" t="n">
-        <v>0.5180952380952381</v>
+        <v>0.5771428571428572</v>
       </c>
       <c r="N2" t="n">
-        <v>0.06305883945617841</v>
+        <v>0.02138089935299395</v>
       </c>
       <c r="O2" t="n">
-        <v>0.589047619047619</v>
+        <v>0.5871428571428571</v>
       </c>
       <c r="P2" t="n">
-        <v>0.036934703675553</v>
+        <v>0.03510915922127</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.0705635110380798</v>
+        <v>0.07613819561276439</v>
       </c>
       <c r="R2" t="n">
-        <v>0.0190063812347331</v>
+        <v>0.01198908252157456</v>
       </c>
       <c r="S2" t="n">
-        <v>0.1072398813531055</v>
+        <v>0.1179061987040757</v>
       </c>
       <c r="T2" t="n">
-        <v>0.021920256908645</v>
+        <v>0.01712355596962507</v>
       </c>
       <c r="U2" t="n">
-        <v>0.2503991631249481</v>
+        <v>0.2478846906692992</v>
       </c>
       <c r="V2" t="n">
-        <v>0.0383648971731178</v>
+        <v>0.04073378046629857</v>
       </c>
       <c r="W2" t="n">
-        <v>0.7308707943419576</v>
+        <v>0.7835082374698987</v>
       </c>
       <c r="X2" t="n">
-        <v>0.0597026467533132</v>
+        <v>0.06641186043717788</v>
       </c>
       <c r="Y2" t="n">
-        <v>0.7764524657154872</v>
+        <v>0.8123186909264417</v>
       </c>
       <c r="Z2" t="n">
-        <v>0.0298205776209729</v>
+        <v>0.03598664275637017</v>
       </c>
       <c r="AA2" t="n">
-        <v>0.7909994976448008</v>
+        <v>0.8126982355860981</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.032176930537804</v>
+        <v>0.02540917232132761</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.8476190476190476</v>
+        <v>0.9428571428571428</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.1060526545300956</v>
+        <v>0.06998542122237654</v>
       </c>
       <c r="AE2" t="n">
-        <v>0.9714285714285716</v>
+        <v>1</v>
       </c>
       <c r="AF2" t="n">
-        <v>0.0571428571428571</v>
+        <v>0</v>
       </c>
       <c r="AG2" t="n">
         <v>1</v>
@@ -730,26 +730,26 @@
         <v>0</v>
       </c>
       <c r="AI2" t="n">
-        <v>0.5453219263336549</v>
+        <v>0.5499564694193888</v>
       </c>
       <c r="AJ2" t="n">
-        <v>0.0146132351062761</v>
+        <v>0.01691237484448266</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>default_none_mse_plain_gat</t>
+          <t>multiple_none_mse_plain_gat</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2_default_relation_baseline</t>
+          <t>1_multi_relation_baseline</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>multiple</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -776,73 +776,73 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>10336.0681912899</v>
+        <v>3092.066526889801</v>
       </c>
       <c r="K3" t="n">
-        <v>0.5904761904761904</v>
+        <v>0.5412698412698413</v>
       </c>
       <c r="L3" t="n">
-        <v>0.0485620906056455</v>
+        <v>0.0869980292447283</v>
       </c>
       <c r="M3" t="n">
-        <v>0.6133333333333334</v>
+        <v>0.5180952380952381</v>
       </c>
       <c r="N3" t="n">
-        <v>0.0484124381986241</v>
+        <v>0.06305883945617841</v>
       </c>
       <c r="O3" t="n">
-        <v>0.5766666666666668</v>
+        <v>0.589047619047619</v>
       </c>
       <c r="P3" t="n">
-        <v>0.0378084442691032</v>
+        <v>0.036934703675553</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.07637005353812069</v>
+        <v>0.0705635110380798</v>
       </c>
       <c r="R3" t="n">
-        <v>0.0156044320746066</v>
+        <v>0.0190063812347331</v>
       </c>
       <c r="S3" t="n">
-        <v>0.1257186444201039</v>
+        <v>0.1072398813531055</v>
       </c>
       <c r="T3" t="n">
-        <v>0.0147868877211523</v>
+        <v>0.021920256908645</v>
       </c>
       <c r="U3" t="n">
-        <v>0.2459841633950435</v>
+        <v>0.2503991631249481</v>
       </c>
       <c r="V3" t="n">
-        <v>0.0414542733808082</v>
+        <v>0.0383648971731178</v>
       </c>
       <c r="W3" t="n">
-        <v>0.8040898926713582</v>
+        <v>0.7308707943419576</v>
       </c>
       <c r="X3" t="n">
-        <v>0.0663045671648796</v>
+        <v>0.0597026467533132</v>
       </c>
       <c r="Y3" t="n">
-        <v>0.8218289172985989</v>
+        <v>0.7764524657154872</v>
       </c>
       <c r="Z3" t="n">
-        <v>0.0292160230826401</v>
+        <v>0.0298205776209729</v>
       </c>
       <c r="AA3" t="n">
-        <v>0.8229725330343598</v>
+        <v>0.7909994976448008</v>
       </c>
       <c r="AB3" t="n">
-        <v>0.02447176407175</v>
+        <v>0.032176930537804</v>
       </c>
       <c r="AC3" t="n">
-        <v>0.9428571428571428</v>
+        <v>0.8476190476190476</v>
       </c>
       <c r="AD3" t="n">
-        <v>0.0699854212223765</v>
+        <v>0.1060526545300956</v>
       </c>
       <c r="AE3" t="n">
-        <v>1</v>
+        <v>0.9714285714285716</v>
       </c>
       <c r="AF3" t="n">
-        <v>0</v>
+        <v>0.0571428571428571</v>
       </c>
       <c r="AG3" t="n">
         <v>1</v>
@@ -851,21 +851,21 @@
         <v>0</v>
       </c>
       <c r="AI3" t="n">
-        <v>0.5474584357147808</v>
+        <v>0.5453219263336549</v>
       </c>
       <c r="AJ3" t="n">
-        <v>0.0164952756099014</v>
+        <v>0.0146132351062761</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>default_causal_fs0_mse_plain_gat</t>
+          <t>default_none_mse_plain_gat</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>3_CE_over_default</t>
+          <t>2_default_relation_baseline</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -875,11 +875,8 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>causal</t>
-        </is>
-      </c>
-      <c r="E4" t="b">
-        <v>0</v>
+          <t>none</t>
+        </is>
       </c>
       <c r="F4" t="b">
         <v>1</v>
@@ -900,67 +897,67 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>8671.333433628082</v>
+        <v>10336.0681912899</v>
       </c>
       <c r="K4" t="n">
-        <v>0.6174603174603175</v>
+        <v>0.5904761904761904</v>
       </c>
       <c r="L4" t="n">
-        <v>0.09040654518030559</v>
+        <v>0.0485620906056455</v>
       </c>
       <c r="M4" t="n">
-        <v>0.6352380952380952</v>
+        <v>0.6133333333333334</v>
       </c>
       <c r="N4" t="n">
-        <v>0.0753284568887054</v>
+        <v>0.0484124381986241</v>
       </c>
       <c r="O4" t="n">
-        <v>0.589047619047619</v>
+        <v>0.5766666666666668</v>
       </c>
       <c r="P4" t="n">
-        <v>0.0562146840509474</v>
+        <v>0.0378084442691032</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.0865512264039464</v>
+        <v>0.07637005353812069</v>
       </c>
       <c r="R4" t="n">
-        <v>0.0263471170360798</v>
+        <v>0.0156044320746066</v>
       </c>
       <c r="S4" t="n">
-        <v>0.1362739817065336</v>
+        <v>0.1257186444201039</v>
       </c>
       <c r="T4" t="n">
-        <v>0.0269848473446352</v>
+        <v>0.0147868877211523</v>
       </c>
       <c r="U4" t="n">
-        <v>0.2452945582600602</v>
+        <v>0.2459841633950435</v>
       </c>
       <c r="V4" t="n">
-        <v>0.0375372441117505</v>
+        <v>0.0414542733808082</v>
       </c>
       <c r="W4" t="n">
-        <v>0.8353965419886867</v>
+        <v>0.8040898926713582</v>
       </c>
       <c r="X4" t="n">
-        <v>0.0675252737111041</v>
+        <v>0.0663045671648796</v>
       </c>
       <c r="Y4" t="n">
-        <v>0.8341328555651175</v>
+        <v>0.8218289172985989</v>
       </c>
       <c r="Z4" t="n">
-        <v>0.0487252230384082</v>
+        <v>0.0292160230826401</v>
       </c>
       <c r="AA4" t="n">
-        <v>0.8312633368724764</v>
+        <v>0.8229725330343598</v>
       </c>
       <c r="AB4" t="n">
-        <v>0.0362133363099123</v>
+        <v>0.02447176407175</v>
       </c>
       <c r="AC4" t="n">
-        <v>0.9714285714285716</v>
+        <v>0.9428571428571428</v>
       </c>
       <c r="AD4" t="n">
-        <v>0.0571428571428571</v>
+        <v>0.0699854212223765</v>
       </c>
       <c r="AE4" t="n">
         <v>1</v>
@@ -975,12 +972,261 @@
         <v>0</v>
       </c>
       <c r="AI4" t="n">
+        <v>0.5474584357147808</v>
+      </c>
+      <c r="AJ4" t="n">
+        <v>0.0164952756099014</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>default_causal_fs0_mse_plain_gat</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>3_CE_over_default</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>causal</t>
+        </is>
+      </c>
+      <c r="E5" t="b">
+        <v>0</v>
+      </c>
+      <c r="F5" t="b">
+        <v>1</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>mse</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>plain</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>gat</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>8671.333433628082</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.6174603174603175</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.09040654518030559</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.6352380952380952</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0.0753284568887054</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0.589047619047619</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0.0562146840509474</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0.0865512264039464</v>
+      </c>
+      <c r="R5" t="n">
+        <v>0.0263471170360798</v>
+      </c>
+      <c r="S5" t="n">
+        <v>0.1362739817065336</v>
+      </c>
+      <c r="T5" t="n">
+        <v>0.0269848473446352</v>
+      </c>
+      <c r="U5" t="n">
+        <v>0.2452945582600602</v>
+      </c>
+      <c r="V5" t="n">
+        <v>0.0375372441117505</v>
+      </c>
+      <c r="W5" t="n">
+        <v>0.8353965419886867</v>
+      </c>
+      <c r="X5" t="n">
+        <v>0.0675252737111041</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>0.8341328555651175</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>0.0487252230384082</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>0.8312633368724764</v>
+      </c>
+      <c r="AB5" t="n">
+        <v>0.0362133363099123</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>0.9714285714285716</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>0.0571428571428571</v>
+      </c>
+      <c r="AE5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI5" t="n">
         <v>0.54924461055519</v>
       </c>
-      <c r="AJ4" t="n">
+      <c r="AJ5" t="n">
         <v>0.0197360384520377</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>default_ace_learnable_fs1_mse_plain_gat</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>4_ACE_over_default</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>ace_learnable</t>
+        </is>
+      </c>
+      <c r="E6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F6" t="b">
+        <v>1</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>mse</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>plain</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>gat</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>13969.57676362991</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.5603174603174603</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.05396825396825398</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0.5542857142857143</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0.05883217223421137</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0.5852380952380953</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0.04334118191612481</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>0.07324442271899148</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0.01602985299789608</v>
+      </c>
+      <c r="S6" t="n">
+        <v>0.1135341518278272</v>
+      </c>
+      <c r="T6" t="n">
+        <v>0.01765719108701027</v>
+      </c>
+      <c r="U6" t="n">
+        <v>0.2500660161827787</v>
+      </c>
+      <c r="V6" t="n">
+        <v>0.03997774755142271</v>
+      </c>
+      <c r="W6" t="n">
+        <v>0.749066205982466</v>
+      </c>
+      <c r="X6" t="n">
+        <v>0.07610617788269321</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>0.8101637387292108</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>0.03418990414937448</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>0.8032817378746273</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>0.01946716098073919</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>0.8761904761904763</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>0.1227057021592869</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI6" t="n">
+        <v>0.5420111819237873</v>
+      </c>
+      <c r="AJ6" t="n">
+        <v>0.01768087693496134</v>
+      </c>
+    </row>
+    <row r="7"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -992,7 +1238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ4"/>
+  <dimension ref="A1:AJ6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1180,17 +1426,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>multiple_none_mse_norm_gcn</t>
+          <t>single_none_mse_norm_gcn</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1_multi_relation_baseline</t>
+          <t>0_single_relation_baseline</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>multiple</t>
+          <t>single</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1217,73 +1463,73 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>4578.097548484802</v>
+        <v>682.2839343547821</v>
       </c>
       <c r="K2" t="n">
-        <v>0.5222222222222223</v>
+        <v>0.5476190476190477</v>
       </c>
       <c r="L2" t="n">
-        <v>0.0651374112021688</v>
+        <v>0.0301169300968417</v>
       </c>
       <c r="M2" t="n">
-        <v>0.5580952380952381</v>
+        <v>0.5866666666666667</v>
       </c>
       <c r="N2" t="n">
-        <v>0.0304761904761904</v>
+        <v>0.0322124467148338</v>
       </c>
       <c r="O2" t="n">
-        <v>0.5771428571428572</v>
+        <v>0.5947619047619048</v>
       </c>
       <c r="P2" t="n">
-        <v>0.0193780856660722</v>
+        <v>0.02975333209869204</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.06835262668433829</v>
+        <v>0.07254055376700223</v>
       </c>
       <c r="R2" t="n">
-        <v>0.0190865840321664</v>
+        <v>0.01649827280107199</v>
       </c>
       <c r="S2" t="n">
-        <v>0.1225422456554698</v>
+        <v>0.1210102005387277</v>
       </c>
       <c r="T2" t="n">
-        <v>0.0331875786619627</v>
+        <v>0.01583799070525876</v>
       </c>
       <c r="U2" t="n">
-        <v>0.2463068595368462</v>
+        <v>0.2533546929752148</v>
       </c>
       <c r="V2" t="n">
-        <v>0.0402503715543969</v>
+        <v>0.03515598093899076</v>
       </c>
       <c r="W2" t="n">
-        <v>0.6976194304709546</v>
+        <v>0.751163036876847</v>
       </c>
       <c r="X2" t="n">
-        <v>0.0223545807761463</v>
+        <v>0.03201164474321516</v>
       </c>
       <c r="Y2" t="n">
-        <v>0.7559797966591107</v>
+        <v>0.7934135774224135</v>
       </c>
       <c r="Z2" t="n">
-        <v>0.0439872876800495</v>
+        <v>0.01861693517472711</v>
       </c>
       <c r="AA2" t="n">
-        <v>0.7856097617635172</v>
+        <v>0.7936120503395421</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.0227980125573923</v>
+        <v>0.01237515561979637</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.8476190476190476</v>
+        <v>0.9428571428571428</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.1060526545300956</v>
+        <v>0.06998542122237654</v>
       </c>
       <c r="AE2" t="n">
-        <v>0.9714285714285716</v>
+        <v>1</v>
       </c>
       <c r="AF2" t="n">
-        <v>0.0571428571428571</v>
+        <v>0</v>
       </c>
       <c r="AG2" t="n">
         <v>1</v>
@@ -1292,26 +1538,26 @@
         <v>0</v>
       </c>
       <c r="AI2" t="n">
-        <v>0.5389895088905609</v>
+        <v>0.5480193259840089</v>
       </c>
       <c r="AJ2" t="n">
-        <v>0.0264913217131037</v>
+        <v>0.01915818045337209</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>default_none_mse_norm_gcn</t>
+          <t>multiple_none_mse_norm_gcn</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2_default_relation_baseline</t>
+          <t>1_multi_relation_baseline</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>multiple</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1338,73 +1584,73 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>14738.54326796532</v>
+        <v>4578.097548484802</v>
       </c>
       <c r="K3" t="n">
-        <v>0.5888888888888889</v>
+        <v>0.5222222222222223</v>
       </c>
       <c r="L3" t="n">
-        <v>0.047724750407533</v>
+        <v>0.0651374112021688</v>
       </c>
       <c r="M3" t="n">
-        <v>0.5952380952380952</v>
+        <v>0.5580952380952381</v>
       </c>
       <c r="N3" t="n">
-        <v>0.0498523898221043</v>
+        <v>0.0304761904761904</v>
       </c>
       <c r="O3" t="n">
-        <v>0.5938095238095238</v>
+        <v>0.5771428571428572</v>
       </c>
       <c r="P3" t="n">
-        <v>0.0281557057125609</v>
+        <v>0.0193780856660722</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.07794157975626349</v>
+        <v>0.06835262668433829</v>
       </c>
       <c r="R3" t="n">
-        <v>0.0156092257695876</v>
+        <v>0.0190865840321664</v>
       </c>
       <c r="S3" t="n">
-        <v>0.1231952328962501</v>
+        <v>0.1225422456554698</v>
       </c>
       <c r="T3" t="n">
-        <v>0.009913983991402701</v>
+        <v>0.0331875786619627</v>
       </c>
       <c r="U3" t="n">
-        <v>0.253495922116444</v>
+        <v>0.2463068595368462</v>
       </c>
       <c r="V3" t="n">
-        <v>0.0369562828142367</v>
+        <v>0.0402503715543969</v>
       </c>
       <c r="W3" t="n">
-        <v>0.6960952109732976</v>
+        <v>0.6976194304709546</v>
       </c>
       <c r="X3" t="n">
-        <v>0.054067638612862</v>
+        <v>0.0223545807761463</v>
       </c>
       <c r="Y3" t="n">
-        <v>0.7854617748166512</v>
+        <v>0.7559797966591107</v>
       </c>
       <c r="Z3" t="n">
-        <v>0.0180244408072348</v>
+        <v>0.0439872876800495</v>
       </c>
       <c r="AA3" t="n">
-        <v>0.8047271213857116</v>
+        <v>0.7856097617635172</v>
       </c>
       <c r="AB3" t="n">
-        <v>0.0112979114540867</v>
+        <v>0.0227980125573923</v>
       </c>
       <c r="AC3" t="n">
-        <v>0.8190476190476191</v>
+        <v>0.8476190476190476</v>
       </c>
       <c r="AD3" t="n">
-        <v>0.1181873680570557</v>
+        <v>0.1060526545300956</v>
       </c>
       <c r="AE3" t="n">
-        <v>1</v>
+        <v>0.9714285714285716</v>
       </c>
       <c r="AF3" t="n">
-        <v>0</v>
+        <v>0.0571428571428571</v>
       </c>
       <c r="AG3" t="n">
         <v>1</v>
@@ -1413,21 +1659,21 @@
         <v>0</v>
       </c>
       <c r="AI3" t="n">
-        <v>0.5461490348774837</v>
+        <v>0.5389895088905609</v>
       </c>
       <c r="AJ3" t="n">
-        <v>0.0231214236938108</v>
+        <v>0.0264913217131037</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>default_ace_learnable_fs1_mse_norm_gcn</t>
+          <t>default_none_mse_norm_gcn</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>3_ACE_over_default</t>
+          <t>2_default_relation_baseline</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1437,11 +1683,8 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>ace_learnable</t>
-        </is>
-      </c>
-      <c r="E4" t="b">
-        <v>1</v>
+          <t>none</t>
+        </is>
       </c>
       <c r="F4" t="b">
         <v>1</v>
@@ -1462,73 +1705,73 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>20137.12212610245</v>
+        <v>14738.54326796532</v>
       </c>
       <c r="K4" t="n">
-        <v>0.619047619047619</v>
+        <v>0.5888888888888889</v>
       </c>
       <c r="L4" t="n">
-        <v>0.0301169300968417</v>
+        <v>0.047724750407533</v>
       </c>
       <c r="M4" t="n">
-        <v>0.5952380952380951</v>
+        <v>0.5952380952380952</v>
       </c>
       <c r="N4" t="n">
-        <v>0.029199447079535</v>
+        <v>0.0498523898221043</v>
       </c>
       <c r="O4" t="n">
-        <v>0.6028571428571429</v>
+        <v>0.5938095238095238</v>
       </c>
       <c r="P4" t="n">
-        <v>0.0277010277566647</v>
+        <v>0.0281557057125609</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.0801789167963427</v>
+        <v>0.07794157975626349</v>
       </c>
       <c r="R4" t="n">
-        <v>0.0127267357191036</v>
+        <v>0.0156092257695876</v>
       </c>
       <c r="S4" t="n">
-        <v>0.1227674936494042</v>
+        <v>0.1231952328962501</v>
       </c>
       <c r="T4" t="n">
-        <v>0.0104981703176155</v>
+        <v>0.009913983991402701</v>
       </c>
       <c r="U4" t="n">
-        <v>0.2551722216879227</v>
+        <v>0.253495922116444</v>
       </c>
       <c r="V4" t="n">
-        <v>0.0365086321136545</v>
+        <v>0.0369562828142367</v>
       </c>
       <c r="W4" t="n">
-        <v>0.7961771804356279</v>
+        <v>0.6960952109732976</v>
       </c>
       <c r="X4" t="n">
-        <v>0.0747823420332452</v>
+        <v>0.054067638612862</v>
       </c>
       <c r="Y4" t="n">
-        <v>0.8073800991577675</v>
+        <v>0.7854617748166512</v>
       </c>
       <c r="Z4" t="n">
-        <v>0.0532421491481552</v>
+        <v>0.0180244408072348</v>
       </c>
       <c r="AA4" t="n">
-        <v>0.8217317668653031</v>
+        <v>0.8047271213857116</v>
       </c>
       <c r="AB4" t="n">
-        <v>0.0225727270255516</v>
+        <v>0.0112979114540867</v>
       </c>
       <c r="AC4" t="n">
-        <v>0.9428571428571428</v>
+        <v>0.8190476190476191</v>
       </c>
       <c r="AD4" t="n">
-        <v>0.0699854212223765</v>
+        <v>0.1181873680570557</v>
       </c>
       <c r="AE4" t="n">
-        <v>0.9714285714285716</v>
+        <v>1</v>
       </c>
       <c r="AF4" t="n">
-        <v>0.0571428571428571</v>
+        <v>0</v>
       </c>
       <c r="AG4" t="n">
         <v>1</v>
@@ -1537,9 +1780,257 @@
         <v>0</v>
       </c>
       <c r="AI4" t="n">
+        <v>0.5461490348774837</v>
+      </c>
+      <c r="AJ4" t="n">
+        <v>0.0231214236938108</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>default_causal_fs0_mse_norm_gcn</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>3_CE_over_default</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>causal</t>
+        </is>
+      </c>
+      <c r="E5" t="b">
+        <v>0</v>
+      </c>
+      <c r="F5" t="b">
+        <v>1</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>mse</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>norm</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>gcn</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>8562.524777889252</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.5603174603174603</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.05396825396825394</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.5666666666666667</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0.04343525428949098</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0.589047619047619</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0.03908244672130133</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0.07256402514385707</v>
+      </c>
+      <c r="R5" t="n">
+        <v>0.01661748726218318</v>
+      </c>
+      <c r="S5" t="n">
+        <v>0.1240698133258947</v>
+      </c>
+      <c r="T5" t="n">
+        <v>0.02979229620476089</v>
+      </c>
+      <c r="U5" t="n">
+        <v>0.2506460259644691</v>
+      </c>
+      <c r="V5" t="n">
+        <v>0.04061695912572197</v>
+      </c>
+      <c r="W5" t="n">
+        <v>0.7631192382554693</v>
+      </c>
+      <c r="X5" t="n">
+        <v>0.06656449920931359</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>0.7971618568029034</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>0.03574486375442113</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>0.7975059854921224</v>
+      </c>
+      <c r="AB5" t="n">
+        <v>0.0271458716149667</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>0.9142857142857143</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>0.1142857142857143</v>
+      </c>
+      <c r="AE5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI5" t="n">
+        <v>0.5479601950288261</v>
+      </c>
+      <c r="AJ5" t="n">
+        <v>0.01975831180494288</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>default_ace_learnable_fs1_mse_norm_gcn</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>4_ACE_over_default</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>ace_learnable</t>
+        </is>
+      </c>
+      <c r="E6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F6" t="b">
+        <v>1</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>mse</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>norm</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>gcn</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>20137.12212610245</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.619047619047619</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.0301169300968417</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0.5952380952380951</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0.029199447079535</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0.6028571428571429</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0.0277010277566647</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>0.0801789167963427</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0.0127267357191036</v>
+      </c>
+      <c r="S6" t="n">
+        <v>0.1227674936494042</v>
+      </c>
+      <c r="T6" t="n">
+        <v>0.0104981703176155</v>
+      </c>
+      <c r="U6" t="n">
+        <v>0.2551722216879227</v>
+      </c>
+      <c r="V6" t="n">
+        <v>0.0365086321136545</v>
+      </c>
+      <c r="W6" t="n">
+        <v>0.7961771804356279</v>
+      </c>
+      <c r="X6" t="n">
+        <v>0.0747823420332452</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>0.8073800991577675</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>0.0532421491481552</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>0.8217317668653031</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>0.0225727270255516</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>0.9428571428571428</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>0.0699854212223765</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>0.9714285714285716</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>0.0571428571428571</v>
+      </c>
+      <c r="AG6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI6" t="n">
         <v>0.5493230017429565</v>
       </c>
-      <c r="AJ4" t="n">
+      <c r="AJ6" t="n">
         <v>0.0185542211322056</v>
       </c>
     </row>

</xml_diff>